<commit_message>
Modificaciones para poder extraer la informacion de el supervisor tecnico
</commit_message>
<xml_diff>
--- a/backend/templates/SCPM-05A.xlsx
+++ b/backend/templates/SCPM-05A.xlsx
@@ -1615,11 +1615,16 @@
       </c>
       <c r="J10" s="102" t="n"/>
       <c r="K10" s="102" t="n"/>
-      <c r="L10" s="102" t="n"/>
-      <c r="M10" s="102" t="n"/>
-      <c r="N10" s="102" t="n"/>
-      <c r="O10" s="102" t="n"/>
-      <c r="P10" s="102" t="n"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Nivel:</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>{{ nivel }}</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -2133,7 +2138,7 @@
       <c r="P37" s="106" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="35">
+  <mergeCells count="36">
     <mergeCell ref="L7:P7"/>
     <mergeCell ref="A37:F37"/>
     <mergeCell ref="J4:L4"/>
@@ -2151,6 +2156,7 @@
     <mergeCell ref="O22:P22"/>
     <mergeCell ref="M13:N13"/>
     <mergeCell ref="M5:P5"/>
+    <mergeCell ref="I10:K10"/>
     <mergeCell ref="K37:P37"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="C4:F4"/>
@@ -2159,12 +2165,12 @@
     <mergeCell ref="C11:G11"/>
     <mergeCell ref="A15:C15"/>
     <mergeCell ref="A34:F36"/>
+    <mergeCell ref="M10:P10"/>
     <mergeCell ref="G37:J37"/>
     <mergeCell ref="E13:H13"/>
     <mergeCell ref="K34:P36"/>
     <mergeCell ref="J5:L5"/>
     <mergeCell ref="C9:F9"/>
-    <mergeCell ref="I10:P10"/>
     <mergeCell ref="G34:J36"/>
     <mergeCell ref="I9:P9"/>
     <mergeCell ref="O13:P13"/>

</xml_diff>